<commit_message>
Add PEP 257 docstrings to class and functions and align code with PEP-8 standards
</commit_message>
<xml_diff>
--- a/spase_helio_compare/excel/all_helioData_spase_names.xlsx
+++ b/spase_helio_compare/excel/all_helioData_spase_names.xlsx
@@ -424,17 +424,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>SPASE_ResourceName</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>HelioData_long_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>SPASE_AlternateName</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>SPASE_ResourceName</t>
         </is>
       </c>
     </row>

</xml_diff>